<commit_message>
Add Class 5 NCERT syllabus Excel in the same import format as Class 4.
Includes Joyful Mathematics chapter names, NCERT chapter column, updated templates, and import tests.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/public/samples/syllabus-import/CBSE_Class5_Maths_Syllabus_TEMPLATE.xlsx
+++ b/public/samples/syllabus-import/CBSE_Class5_Maths_Syllabus_TEMPLATE.xlsx
@@ -7,7 +7,7 @@
     <workbookView activeTab="0" autoFilterDateGrouping="true" firstSheet="0" minimized="false" showHorizontalScroll="true" showSheetTabs="true" showVerticalScroll="true" tabRatio="600" visibility="visible"/>
   </bookViews>
   <sheets>
-    <sheet name="Syllabus" sheetId="1" r:id="rId4"/>
+    <sheet name="Class 5 Syllabus" sheetId="1" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="999999" calcMode="auto" calcCompleted="1" fullCalcOnLoad="0" forceFullCalc="0"/>
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="119">
   <si>
     <t>Chapter No.</t>
   </si>
@@ -23,67 +23,355 @@
     <t>Main Topic (Chapter)</t>
   </si>
   <si>
+    <t xml:space="preserve">chapter </t>
+  </si>
+  <si>
     <t>Sub-Topic</t>
   </si>
   <si>
     <t>Key Concepts / Learning Outcomes</t>
   </si>
   <si>
-    <t>Difficulty Level</t>
-  </si>
-  <si>
     <t>Approx. Periods</t>
   </si>
   <si>
     <t>Remarks</t>
   </si>
   <si>
-    <t>The Fish Tale</t>
-  </si>
-  <si>
-    <t>Large numbers in real life</t>
-  </si>
-  <si>
-    <t>Read and write numbers beyond 10000</t>
-  </si>
-  <si>
-    <t>Easy</t>
-  </si>
-  <si>
-    <t>NCERT Ch 1 — replace with official CBSE syllabus</t>
-  </si>
-  <si>
-    <t>Shapes and Angles</t>
-  </si>
-  <si>
-    <t>Types of angles</t>
-  </si>
-  <si>
-    <t>Identify acute, right, obtuse angles</t>
-  </si>
-  <si>
-    <t>NCERT Ch 2</t>
-  </si>
-  <si>
-    <t>Measuring angles</t>
-  </si>
-  <si>
-    <t>Use protractor; estimate angle size</t>
-  </si>
-  <si>
-    <t>Medium</t>
-  </si>
-  <si>
-    <t>How Many Squares?</t>
-  </si>
-  <si>
-    <t>Area by counting squares</t>
-  </si>
-  <si>
-    <t>Find area on grid paper</t>
-  </si>
-  <si>
-    <t>NCERT Ch 3 — sample only</t>
+    <t>Number System</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> We the Travellers—I</t>
+  </si>
+  <si>
+    <t>Large Numbers in Travel</t>
+  </si>
+  <si>
+    <t>Reading and writing numbers up to lakhs in journey contexts</t>
+  </si>
+  <si>
+    <t>NCERT opening chapter</t>
+  </si>
+  <si>
+    <t>Routes and Distances</t>
+  </si>
+  <si>
+    <t>Interpreting route charts, comparing distances between places</t>
+  </si>
+  <si>
+    <t>Planning a Journey</t>
+  </si>
+  <si>
+    <t>Estimating cost, time and resources for a trip</t>
+  </si>
+  <si>
+    <t>Ratio &amp; Proportion</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Fractions</t>
+  </si>
+  <si>
+    <t>Unit and Like Fractions</t>
+  </si>
+  <si>
+    <t>Understanding numerator, denominator and equal parts of a whole</t>
+  </si>
+  <si>
+    <t>Equivalent Fractions</t>
+  </si>
+  <si>
+    <t>Finding equal fractions using models and multiplication</t>
+  </si>
+  <si>
+    <t>Comparing Fractions</t>
+  </si>
+  <si>
+    <t>Ordering fractions with same denominator or using benchmarks</t>
+  </si>
+  <si>
+    <t>Geometry</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Angles as Turns</t>
+  </si>
+  <si>
+    <t>Turns as Fractions of a Circle</t>
+  </si>
+  <si>
+    <t>Full, half, quarter and three-quarter turns</t>
+  </si>
+  <si>
+    <t>Measuring Turns</t>
+  </si>
+  <si>
+    <t>Relating turns to right angles and everyday rotation</t>
+  </si>
+  <si>
+    <t>Angles in Movement</t>
+  </si>
+  <si>
+    <t>Describing direction change using turn language</t>
+  </si>
+  <si>
+    <t>Speed Distance Time</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> We the Travellers—II</t>
+  </si>
+  <si>
+    <t>Reading Timetables</t>
+  </si>
+  <si>
+    <t>Using bus and train schedules to plan travel</t>
+  </si>
+  <si>
+    <t>Distance and Time Estimates</t>
+  </si>
+  <si>
+    <t>Linking speed, distance and time in simple situations</t>
+  </si>
+  <si>
+    <t>Multi-step Travel Problems</t>
+  </si>
+  <si>
+    <t>Addition and subtraction in route-planning contexts</t>
+  </si>
+  <si>
+    <t>Perimeter and Area</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Far and Near</t>
+  </si>
+  <si>
+    <t>Comparing Distances</t>
+  </si>
+  <si>
+    <t>Near/far, longer/shorter using non-standard units</t>
+  </si>
+  <si>
+    <t>Standard Units of Length</t>
+  </si>
+  <si>
+    <t>Using cm, m and km with rulers and measuring tapes</t>
+  </si>
+  <si>
+    <t>Length Word Problems</t>
+  </si>
+  <si>
+    <t>Addition and subtraction problems involving distance</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> The Dairy Farm</t>
+  </si>
+  <si>
+    <t>Multiplication in Farming</t>
+  </si>
+  <si>
+    <t>Equal groups, arrays and repeated addition for milk yield</t>
+  </si>
+  <si>
+    <t>Division and Sharing</t>
+  </si>
+  <si>
+    <t>Sharing produce equally among workers or containers</t>
+  </si>
+  <si>
+    <t>Farm Budget Problems</t>
+  </si>
+  <si>
+    <t>Simple cost and quantity problems in a dairy setting</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Shapes and Patterns</t>
+  </si>
+  <si>
+    <t>2D Shapes and Properties</t>
+  </si>
+  <si>
+    <t>Identifying sides, corners and names of common shapes</t>
+  </si>
+  <si>
+    <t>Tessellations and Tiling</t>
+  </si>
+  <si>
+    <t>Repeating shapes to cover a surface without gaps</t>
+  </si>
+  <si>
+    <t>Creating Shape Patterns</t>
+  </si>
+  <si>
+    <t>Designing borders, rangoli and repeating motifs</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Weight and Capacity</t>
+  </si>
+  <si>
+    <t>Kilograms and Grams</t>
+  </si>
+  <si>
+    <t>Weighing objects and converting between kg and g</t>
+  </si>
+  <si>
+    <t>Litres and Millilitres</t>
+  </si>
+  <si>
+    <t>Measuring liquids and reading capacity scales</t>
+  </si>
+  <si>
+    <t>Weight and Capacity Problems</t>
+  </si>
+  <si>
+    <t>Applied problems on shopping and cooking quantities</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Coconut Farm</t>
+  </si>
+  <si>
+    <t>Fractions of a Harvest</t>
+  </si>
+  <si>
+    <t>Finding half, third or quarter of a collection of coconuts</t>
+  </si>
+  <si>
+    <t>Equal Sharing on the Farm</t>
+  </si>
+  <si>
+    <t>Division and grouping in harvesting and packing contexts</t>
+  </si>
+  <si>
+    <t>Farm Income Problems</t>
+  </si>
+  <si>
+    <t>Simple profit and sharing problems using fractions</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Symmetrical Designs</t>
+  </si>
+  <si>
+    <t>Line Symmetry</t>
+  </si>
+  <si>
+    <t>Identifying lines of symmetry in shapes and letters</t>
+  </si>
+  <si>
+    <t>Completing Symmetric Figures</t>
+  </si>
+  <si>
+    <t>Drawing mirror halves of patterns and objects</t>
+  </si>
+  <si>
+    <t>Symmetry in Art</t>
+  </si>
+  <si>
+    <t>Creating symmetric rangoli, kolam and craft designs</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Grandmother's Quilt</t>
+  </si>
+  <si>
+    <t>Patchwork Patterns</t>
+  </si>
+  <si>
+    <t>Arranging coloured squares and triangles on a grid</t>
+  </si>
+  <si>
+    <t>Fractions on a Quilt</t>
+  </si>
+  <si>
+    <t>Shading fractional parts of a patchwork layout</t>
+  </si>
+  <si>
+    <t>Designing a Quilt Plan</t>
+  </si>
+  <si>
+    <t>Planning rows, columns and repeating colour blocks</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Racing Seconds</t>
+  </si>
+  <si>
+    <t>Reading Time to the Second</t>
+  </si>
+  <si>
+    <t>Using clocks and stopwatches with seconds</t>
+  </si>
+  <si>
+    <t>Comparing Race Times</t>
+  </si>
+  <si>
+    <t>Finding faster/slower by comparing mm:ss readings</t>
+  </si>
+  <si>
+    <t>Elapsed Time Problems</t>
+  </si>
+  <si>
+    <t>Calculating time taken in short-duration events</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Animal Jumps</t>
+  </si>
+  <si>
+    <t>Measuring Jump Lengths</t>
+  </si>
+  <si>
+    <t>Recording how far animals jump using standard units</t>
+  </si>
+  <si>
+    <t>Comparing and Ordering Lengths</t>
+  </si>
+  <si>
+    <t>Ranking jump data from shortest to longest</t>
+  </si>
+  <si>
+    <t>Average Jump (Intro)</t>
+  </si>
+  <si>
+    <t>Finding a typical jump length from a small data set</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Maps and Locations</t>
+  </si>
+  <si>
+    <t>Grid References</t>
+  </si>
+  <si>
+    <t>Locating places using row–column grids on maps</t>
+  </si>
+  <si>
+    <t>Cardinal Directions</t>
+  </si>
+  <si>
+    <t>North, south, east, west and relative position</t>
+  </si>
+  <si>
+    <t>Scale and Distance on Maps</t>
+  </si>
+  <si>
+    <t>Simple scale reading (e.g. 1 cm = 1 km)</t>
+  </si>
+  <si>
+    <t>Statistics</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Data Through Pictures</t>
+  </si>
+  <si>
+    <t>Collecting and Tallying Data</t>
+  </si>
+  <si>
+    <t>Recording observations using tally marks</t>
+  </si>
+  <si>
+    <t>Pictographs</t>
+  </si>
+  <si>
+    <t>Representing data with symbols and a scale</t>
+  </si>
+  <si>
+    <t>Reading Bar Graphs</t>
+  </si>
+  <si>
+    <t>Answering questions from bar charts and pictures</t>
   </si>
 </sst>
 </file>
@@ -423,16 +711,16 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:G5"/>
+  <dimension ref="A1:G46"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" width="13.997" bestFit="true" customWidth="true" style="0"/>
     <col min="2" max="2" width="24.708" bestFit="true" customWidth="true" style="0"/>
-    <col min="3" max="3" width="31.707" bestFit="true" customWidth="true" style="0"/>
-    <col min="4" max="4" width="43.561" bestFit="true" customWidth="true" style="0"/>
-    <col min="5" max="5" width="19.995" bestFit="true" customWidth="true" style="0"/>
+    <col min="3" max="3" width="26.993" bestFit="true" customWidth="true" style="0"/>
+    <col min="4" max="4" width="36.42" bestFit="true" customWidth="true" style="0"/>
+    <col min="5" max="5" width="75.41" bestFit="true" customWidth="true" style="0"/>
     <col min="6" max="6" width="18.71" bestFit="true" customWidth="true" style="0"/>
-    <col min="7" max="7" width="57.7" bestFit="true" customWidth="true" style="0"/>
+    <col min="7" max="7" width="25.851" bestFit="true" customWidth="true" style="0"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
@@ -475,7 +763,7 @@
         <v>10</v>
       </c>
       <c r="F2">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="G2" t="s">
         <v>11</v>
@@ -483,68 +771,882 @@
     </row>
     <row r="3" spans="1:7">
       <c r="A3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C3" t="s">
+        <v>8</v>
+      </c>
+      <c r="D3" t="s">
         <v>12</v>
       </c>
-      <c r="C3" t="s">
+      <c r="E3" t="s">
         <v>13</v>
       </c>
-      <c r="D3" t="s">
-        <v>14</v>
-      </c>
-      <c r="E3" t="s">
-        <v>10</v>
-      </c>
       <c r="F3">
-        <v>10</v>
-      </c>
-      <c r="G3" t="s">
-        <v>15</v>
+        <v>3</v>
       </c>
     </row>
     <row r="4" spans="1:7">
       <c r="A4">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B4" t="s">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="C4" t="s">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="D4" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="E4" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="F4">
-        <v>10</v>
+        <v>3</v>
       </c>
     </row>
     <row r="5" spans="1:7">
       <c r="A5">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C5" t="s">
+        <v>17</v>
+      </c>
+      <c r="D5" t="s">
+        <v>18</v>
+      </c>
+      <c r="E5" t="s">
         <v>19</v>
       </c>
-      <c r="C5" t="s">
+      <c r="F5">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7">
+      <c r="A6">
+        <v>2</v>
+      </c>
+      <c r="B6" t="s">
+        <v>16</v>
+      </c>
+      <c r="C6" t="s">
+        <v>17</v>
+      </c>
+      <c r="D6" t="s">
         <v>20</v>
       </c>
-      <c r="D5" t="s">
+      <c r="E6" t="s">
         <v>21</v>
       </c>
-      <c r="E5" t="s">
+      <c r="F6">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7">
+      <c r="A7">
+        <v>2</v>
+      </c>
+      <c r="B7" t="s">
+        <v>16</v>
+      </c>
+      <c r="C7" t="s">
+        <v>17</v>
+      </c>
+      <c r="D7" t="s">
+        <v>22</v>
+      </c>
+      <c r="E7" t="s">
+        <v>23</v>
+      </c>
+      <c r="F7">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7">
+      <c r="A8">
+        <v>3</v>
+      </c>
+      <c r="B8" t="s">
+        <v>24</v>
+      </c>
+      <c r="C8" t="s">
+        <v>25</v>
+      </c>
+      <c r="D8" t="s">
+        <v>26</v>
+      </c>
+      <c r="E8" t="s">
+        <v>27</v>
+      </c>
+      <c r="F8">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7">
+      <c r="A9">
+        <v>3</v>
+      </c>
+      <c r="B9" t="s">
+        <v>24</v>
+      </c>
+      <c r="C9" t="s">
+        <v>25</v>
+      </c>
+      <c r="D9" t="s">
+        <v>28</v>
+      </c>
+      <c r="E9" t="s">
+        <v>29</v>
+      </c>
+      <c r="F9">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7">
+      <c r="A10">
+        <v>3</v>
+      </c>
+      <c r="B10" t="s">
+        <v>24</v>
+      </c>
+      <c r="C10" t="s">
+        <v>25</v>
+      </c>
+      <c r="D10" t="s">
+        <v>30</v>
+      </c>
+      <c r="E10" t="s">
+        <v>31</v>
+      </c>
+      <c r="F10">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7">
+      <c r="A11">
+        <v>4</v>
+      </c>
+      <c r="B11" t="s">
+        <v>32</v>
+      </c>
+      <c r="C11" t="s">
+        <v>33</v>
+      </c>
+      <c r="D11" t="s">
+        <v>34</v>
+      </c>
+      <c r="E11" t="s">
+        <v>35</v>
+      </c>
+      <c r="F11">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7">
+      <c r="A12">
+        <v>4</v>
+      </c>
+      <c r="B12" t="s">
+        <v>32</v>
+      </c>
+      <c r="C12" t="s">
+        <v>33</v>
+      </c>
+      <c r="D12" t="s">
+        <v>36</v>
+      </c>
+      <c r="E12" t="s">
+        <v>37</v>
+      </c>
+      <c r="F12">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7">
+      <c r="A13">
+        <v>4</v>
+      </c>
+      <c r="B13" t="s">
+        <v>32</v>
+      </c>
+      <c r="C13" t="s">
+        <v>33</v>
+      </c>
+      <c r="D13" t="s">
+        <v>38</v>
+      </c>
+      <c r="E13" t="s">
+        <v>39</v>
+      </c>
+      <c r="F13">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7">
+      <c r="A14">
+        <v>5</v>
+      </c>
+      <c r="B14" t="s">
+        <v>40</v>
+      </c>
+      <c r="C14" t="s">
+        <v>41</v>
+      </c>
+      <c r="D14" t="s">
+        <v>42</v>
+      </c>
+      <c r="E14" t="s">
+        <v>43</v>
+      </c>
+      <c r="F14">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7">
+      <c r="A15">
+        <v>5</v>
+      </c>
+      <c r="B15" t="s">
+        <v>40</v>
+      </c>
+      <c r="C15" t="s">
+        <v>41</v>
+      </c>
+      <c r="D15" t="s">
+        <v>44</v>
+      </c>
+      <c r="E15" t="s">
+        <v>45</v>
+      </c>
+      <c r="F15">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7">
+      <c r="A16">
+        <v>5</v>
+      </c>
+      <c r="B16" t="s">
+        <v>40</v>
+      </c>
+      <c r="C16" t="s">
+        <v>41</v>
+      </c>
+      <c r="D16" t="s">
+        <v>46</v>
+      </c>
+      <c r="E16" t="s">
+        <v>47</v>
+      </c>
+      <c r="F16">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7">
+      <c r="A17">
+        <v>6</v>
+      </c>
+      <c r="B17" t="s">
+        <v>7</v>
+      </c>
+      <c r="C17" t="s">
+        <v>48</v>
+      </c>
+      <c r="D17" t="s">
+        <v>49</v>
+      </c>
+      <c r="E17" t="s">
+        <v>50</v>
+      </c>
+      <c r="F17">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7">
+      <c r="A18">
+        <v>6</v>
+      </c>
+      <c r="B18" t="s">
+        <v>7</v>
+      </c>
+      <c r="C18" t="s">
+        <v>48</v>
+      </c>
+      <c r="D18" t="s">
+        <v>51</v>
+      </c>
+      <c r="E18" t="s">
+        <v>52</v>
+      </c>
+      <c r="F18">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7">
+      <c r="A19">
+        <v>6</v>
+      </c>
+      <c r="B19" t="s">
+        <v>7</v>
+      </c>
+      <c r="C19" t="s">
+        <v>48</v>
+      </c>
+      <c r="D19" t="s">
+        <v>53</v>
+      </c>
+      <c r="E19" t="s">
+        <v>54</v>
+      </c>
+      <c r="F19">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7">
+      <c r="A20">
+        <v>7</v>
+      </c>
+      <c r="B20" t="s">
+        <v>24</v>
+      </c>
+      <c r="C20" t="s">
+        <v>55</v>
+      </c>
+      <c r="D20" t="s">
+        <v>56</v>
+      </c>
+      <c r="E20" t="s">
+        <v>57</v>
+      </c>
+      <c r="F20">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7">
+      <c r="A21">
+        <v>7</v>
+      </c>
+      <c r="B21" t="s">
+        <v>24</v>
+      </c>
+      <c r="C21" t="s">
+        <v>55</v>
+      </c>
+      <c r="D21" t="s">
+        <v>58</v>
+      </c>
+      <c r="E21" t="s">
+        <v>59</v>
+      </c>
+      <c r="F21">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7">
+      <c r="A22">
+        <v>7</v>
+      </c>
+      <c r="B22" t="s">
+        <v>24</v>
+      </c>
+      <c r="C22" t="s">
+        <v>55</v>
+      </c>
+      <c r="D22" t="s">
+        <v>60</v>
+      </c>
+      <c r="E22" t="s">
+        <v>61</v>
+      </c>
+      <c r="F22">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7">
+      <c r="A23">
+        <v>8</v>
+      </c>
+      <c r="B23" t="s">
+        <v>40</v>
+      </c>
+      <c r="C23" t="s">
+        <v>62</v>
+      </c>
+      <c r="D23" t="s">
+        <v>63</v>
+      </c>
+      <c r="E23" t="s">
+        <v>64</v>
+      </c>
+      <c r="F23">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7">
+      <c r="A24">
+        <v>8</v>
+      </c>
+      <c r="B24" t="s">
+        <v>40</v>
+      </c>
+      <c r="C24" t="s">
+        <v>62</v>
+      </c>
+      <c r="D24" t="s">
+        <v>65</v>
+      </c>
+      <c r="E24" t="s">
+        <v>66</v>
+      </c>
+      <c r="F24">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7">
+      <c r="A25">
+        <v>8</v>
+      </c>
+      <c r="B25" t="s">
+        <v>40</v>
+      </c>
+      <c r="C25" t="s">
+        <v>62</v>
+      </c>
+      <c r="D25" t="s">
+        <v>67</v>
+      </c>
+      <c r="E25" t="s">
+        <v>68</v>
+      </c>
+      <c r="F25">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7">
+      <c r="A26">
+        <v>9</v>
+      </c>
+      <c r="B26" t="s">
+        <v>16</v>
+      </c>
+      <c r="C26" t="s">
+        <v>69</v>
+      </c>
+      <c r="D26" t="s">
+        <v>70</v>
+      </c>
+      <c r="E26" t="s">
+        <v>71</v>
+      </c>
+      <c r="F26">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7">
+      <c r="A27">
+        <v>9</v>
+      </c>
+      <c r="B27" t="s">
+        <v>16</v>
+      </c>
+      <c r="C27" t="s">
+        <v>69</v>
+      </c>
+      <c r="D27" t="s">
+        <v>72</v>
+      </c>
+      <c r="E27" t="s">
+        <v>73</v>
+      </c>
+      <c r="F27">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7">
+      <c r="A28">
+        <v>9</v>
+      </c>
+      <c r="B28" t="s">
+        <v>16</v>
+      </c>
+      <c r="C28" t="s">
+        <v>69</v>
+      </c>
+      <c r="D28" t="s">
+        <v>74</v>
+      </c>
+      <c r="E28" t="s">
+        <v>75</v>
+      </c>
+      <c r="F28">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7">
+      <c r="A29">
         <v>10</v>
       </c>
-      <c r="F5">
+      <c r="B29" t="s">
+        <v>24</v>
+      </c>
+      <c r="C29" t="s">
+        <v>76</v>
+      </c>
+      <c r="D29" t="s">
+        <v>77</v>
+      </c>
+      <c r="E29" t="s">
+        <v>78</v>
+      </c>
+      <c r="F29">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7">
+      <c r="A30">
+        <v>10</v>
+      </c>
+      <c r="B30" t="s">
+        <v>24</v>
+      </c>
+      <c r="C30" t="s">
+        <v>76</v>
+      </c>
+      <c r="D30" t="s">
+        <v>79</v>
+      </c>
+      <c r="E30" t="s">
+        <v>80</v>
+      </c>
+      <c r="F30">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7">
+      <c r="A31">
+        <v>10</v>
+      </c>
+      <c r="B31" t="s">
+        <v>24</v>
+      </c>
+      <c r="C31" t="s">
+        <v>76</v>
+      </c>
+      <c r="D31" t="s">
+        <v>81</v>
+      </c>
+      <c r="E31" t="s">
+        <v>82</v>
+      </c>
+      <c r="F31">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7">
+      <c r="A32">
+        <v>11</v>
+      </c>
+      <c r="B32" t="s">
+        <v>24</v>
+      </c>
+      <c r="C32" t="s">
+        <v>83</v>
+      </c>
+      <c r="D32" t="s">
+        <v>84</v>
+      </c>
+      <c r="E32" t="s">
+        <v>85</v>
+      </c>
+      <c r="F32">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7">
+      <c r="A33">
+        <v>11</v>
+      </c>
+      <c r="B33" t="s">
+        <v>24</v>
+      </c>
+      <c r="C33" t="s">
+        <v>83</v>
+      </c>
+      <c r="D33" t="s">
+        <v>86</v>
+      </c>
+      <c r="E33" t="s">
+        <v>87</v>
+      </c>
+      <c r="F33">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7">
+      <c r="A34">
+        <v>11</v>
+      </c>
+      <c r="B34" t="s">
+        <v>24</v>
+      </c>
+      <c r="C34" t="s">
+        <v>83</v>
+      </c>
+      <c r="D34" t="s">
+        <v>88</v>
+      </c>
+      <c r="E34" t="s">
+        <v>89</v>
+      </c>
+      <c r="F34">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7">
+      <c r="A35">
         <v>12</v>
       </c>
-      <c r="G5" t="s">
-        <v>22</v>
+      <c r="B35" t="s">
+        <v>32</v>
+      </c>
+      <c r="C35" t="s">
+        <v>90</v>
+      </c>
+      <c r="D35" t="s">
+        <v>91</v>
+      </c>
+      <c r="E35" t="s">
+        <v>92</v>
+      </c>
+      <c r="F35">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7">
+      <c r="A36">
+        <v>12</v>
+      </c>
+      <c r="B36" t="s">
+        <v>32</v>
+      </c>
+      <c r="C36" t="s">
+        <v>90</v>
+      </c>
+      <c r="D36" t="s">
+        <v>93</v>
+      </c>
+      <c r="E36" t="s">
+        <v>94</v>
+      </c>
+      <c r="F36">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7">
+      <c r="A37">
+        <v>12</v>
+      </c>
+      <c r="B37" t="s">
+        <v>32</v>
+      </c>
+      <c r="C37" t="s">
+        <v>90</v>
+      </c>
+      <c r="D37" t="s">
+        <v>95</v>
+      </c>
+      <c r="E37" t="s">
+        <v>96</v>
+      </c>
+      <c r="F37">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7">
+      <c r="A38">
+        <v>13</v>
+      </c>
+      <c r="B38" t="s">
+        <v>40</v>
+      </c>
+      <c r="C38" t="s">
+        <v>97</v>
+      </c>
+      <c r="D38" t="s">
+        <v>98</v>
+      </c>
+      <c r="E38" t="s">
+        <v>99</v>
+      </c>
+      <c r="F38">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7">
+      <c r="A39">
+        <v>13</v>
+      </c>
+      <c r="B39" t="s">
+        <v>40</v>
+      </c>
+      <c r="C39" t="s">
+        <v>97</v>
+      </c>
+      <c r="D39" t="s">
+        <v>100</v>
+      </c>
+      <c r="E39" t="s">
+        <v>101</v>
+      </c>
+      <c r="F39">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7">
+      <c r="A40">
+        <v>13</v>
+      </c>
+      <c r="B40" t="s">
+        <v>40</v>
+      </c>
+      <c r="C40" t="s">
+        <v>97</v>
+      </c>
+      <c r="D40" t="s">
+        <v>102</v>
+      </c>
+      <c r="E40" t="s">
+        <v>103</v>
+      </c>
+      <c r="F40">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7">
+      <c r="A41">
+        <v>14</v>
+      </c>
+      <c r="B41" t="s">
+        <v>24</v>
+      </c>
+      <c r="C41" t="s">
+        <v>104</v>
+      </c>
+      <c r="D41" t="s">
+        <v>105</v>
+      </c>
+      <c r="E41" t="s">
+        <v>106</v>
+      </c>
+      <c r="F41">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7">
+      <c r="A42">
+        <v>14</v>
+      </c>
+      <c r="B42" t="s">
+        <v>24</v>
+      </c>
+      <c r="C42" t="s">
+        <v>104</v>
+      </c>
+      <c r="D42" t="s">
+        <v>107</v>
+      </c>
+      <c r="E42" t="s">
+        <v>108</v>
+      </c>
+      <c r="F42">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="43" spans="1:7">
+      <c r="A43">
+        <v>14</v>
+      </c>
+      <c r="B43" t="s">
+        <v>24</v>
+      </c>
+      <c r="C43" t="s">
+        <v>104</v>
+      </c>
+      <c r="D43" t="s">
+        <v>109</v>
+      </c>
+      <c r="E43" t="s">
+        <v>110</v>
+      </c>
+      <c r="F43">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="44" spans="1:7">
+      <c r="A44">
+        <v>15</v>
+      </c>
+      <c r="B44" t="s">
+        <v>111</v>
+      </c>
+      <c r="C44" t="s">
+        <v>112</v>
+      </c>
+      <c r="D44" t="s">
+        <v>113</v>
+      </c>
+      <c r="E44" t="s">
+        <v>114</v>
+      </c>
+      <c r="F44">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="45" spans="1:7">
+      <c r="A45">
+        <v>15</v>
+      </c>
+      <c r="B45" t="s">
+        <v>111</v>
+      </c>
+      <c r="C45" t="s">
+        <v>112</v>
+      </c>
+      <c r="D45" t="s">
+        <v>115</v>
+      </c>
+      <c r="E45" t="s">
+        <v>116</v>
+      </c>
+      <c r="F45">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="46" spans="1:7">
+      <c r="A46">
+        <v>15</v>
+      </c>
+      <c r="B46" t="s">
+        <v>111</v>
+      </c>
+      <c r="C46" t="s">
+        <v>112</v>
+      </c>
+      <c r="D46" t="s">
+        <v>117</v>
+      </c>
+      <c r="E46" t="s">
+        <v>118</v>
+      </c>
+      <c r="F46">
+        <v>3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>